<commit_message>
Certificate focused learnings added
</commit_message>
<xml_diff>
--- a/Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
+++ b/Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\GITHUB-REPO-SLINK\Kubernetes-Certification-Handson\Certification_Focused_Learnings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D21BADD8-99E7-4445-B35C-AA9DC6774471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB23E08-803D-4144-BBCF-83F2F327997F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="81">
   <si>
     <t>Pod</t>
   </si>
@@ -756,6 +756,9 @@
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="B9" t="s">
+        <v>65</v>
+      </c>
       <c r="C9" t="s">
         <v>79</v>
       </c>

</xml_diff>

<commit_message>
Learned yaml datastructure relationships and model
</commit_message>
<xml_diff>
--- a/Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
+++ b/Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\GITHUB-REPO-SLINK\Kubernetes-Certification-Handson\Certification_Focused_Learnings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB23E08-803D-4144-BBCF-83F2F327997F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562FE7B0-6D28-4646-9EA0-C604E8CD147E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="82">
   <si>
     <t>Pod</t>
   </si>
@@ -311,12 +311,32 @@
   <si>
     <t>generate locally without sending the object to the API server. -o yaml → output the generated resource as YAML. Use &gt; nginx.yaml to save the definition to a file and apply manually using kubectl apply -f  &lt;file name&gt;</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>spec</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is an object containing a container list, and that list contains container objects.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -345,6 +365,13 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -366,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -376,6 +403,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -766,6 +794,11 @@
         <v>80</v>
       </c>
     </row>
+    <row r="10" spans="1:4">
+      <c r="D10" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
     <row r="11" spans="1:4" ht="18">
       <c r="A11" s="1" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Deployment related imperative commands learned
</commit_message>
<xml_diff>
--- a/Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
+++ b/Certification_Focused_Learnings/CKA Learning-Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\GITHUB-REPO-SLINK\Kubernetes-Certification-Handson\Certification_Focused_Learnings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562FE7B0-6D28-4646-9EA0-C604E8CD147E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB701C82-0F91-4D7B-8C57-1443380BAE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="97">
   <si>
     <t>Pod</t>
   </si>
@@ -64,9 +64,6 @@
   </si>
   <si>
     <t>Change Deployment image</t>
-  </si>
-  <si>
-    <t>Generate Deployment YAML</t>
   </si>
   <si>
     <t>Service</t>
@@ -331,12 +328,76 @@
       <t xml:space="preserve"> is an object containing a container list, and that list contains container objects.</t>
     </r>
   </si>
+  <si>
+    <t>kubectl create deployment my-deployment --image=nginx</t>
+  </si>
+  <si>
+    <t>The ReplicaSet is the component maintaining the desired number of Pods. If you do not specify replica, default is 1</t>
+  </si>
+  <si>
+    <t>kubectl create deploy my-deployment --image=nginx --replicas=2</t>
+  </si>
+  <si>
+    <t>replicas determine the desired umber of pods. Kubernetes controller ensure that the desired number is always maintained</t>
+  </si>
+  <si>
+    <t>kubectl create deploy my-deployment --image=nginx --replicas=2 -n test-ns</t>
+  </si>
+  <si>
+    <t>kubectl scale deployment my-deployment --replicas=3  and kubectl scale deployment my-deployment --replicas=2</t>
+  </si>
+  <si>
+    <r>
+      <t>kubectl set image deploymnt my-deployment</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> nginx=nginx:1.27</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve"> nginx=nginx:1.27  means   &lt;container name inside the deployment&gt; = &lt;image nameand tag of that container&gt;</t>
+  </si>
+  <si>
+    <t>Rollouts and history</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kubectl set env deployment my-deployment  APP_ENV=production, </t>
+  </si>
+  <si>
+    <t>kubectl set resources deployment web \
+  --requests=cpu=100m,memory=128Mi \
+  --limits=cpu=500m,memory=256Mi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change Other Deployment paramenters </t>
+  </si>
+  <si>
+    <t>Multi pod deployments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kubectl rollout history deploy  my-deployment, kubectl annoate deployment my-deployment kubernetes.io/change-cause="Updated image to latest", </t>
+  </si>
+  <si>
+    <t>kubernetes.io/change-cause="Updated image to latest" : This is actually a key value pair that is set in the deployment manifest under annotations:
+kubectl rollout specifically look for this key "kubernetes.io/change-cause" and populte the value to the CHANGE-CAUSE field of the rollout history comamnd.</t>
+  </si>
+  <si>
+    <t>There is no imperative command. You have to use the pod manifest to create it.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -364,13 +425,6 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -403,7 +457,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,12 +740,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:D89"/>
+  <dimension ref="A2:D90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.140625" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="71.140625" customWidth="1"/>
+    <col min="3" max="3" width="105.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="110.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -698,13 +754,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -715,13 +771,13 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" t="s">
         <v>65</v>
       </c>
-      <c r="C4" t="s">
-        <v>66</v>
-      </c>
       <c r="D4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -729,13 +785,13 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -743,13 +799,13 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" t="s">
         <v>72</v>
-      </c>
-      <c r="D6" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -757,13 +813,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" t="s">
         <v>74</v>
-      </c>
-      <c r="D7" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -771,13 +827,13 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" t="s">
         <v>76</v>
-      </c>
-      <c r="D8" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -785,18 +841,18 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" t="s">
         <v>79</v>
       </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="10" spans="1:4">
+      <c r="D10" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="D10" s="5" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18">
@@ -811,315 +867,388 @@
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="B13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="B14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="B15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:1">
+      <c r="B16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="18" spans="1:1">
+      <c r="B17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="45">
       <c r="A18" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="75">
+      <c r="A19" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" t="s">
+        <v>94</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="18">
+      <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="18">
-      <c r="A20" s="1" t="s">
+    <row r="22" spans="1:4">
+      <c r="A22" s="2"/>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
-      <c r="A21" s="2"/>
-    </row>
-    <row r="22" spans="1:1">
-      <c r="A22" s="2" t="s">
+    <row r="24" spans="1:4">
+      <c r="A24" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
-      <c r="A23" s="2" t="s">
+    <row r="25" spans="1:4">
+      <c r="A25" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
-      <c r="A24" s="2" t="s">
+    <row r="26" spans="1:4">
+      <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
-      <c r="A25" s="2" t="s">
+    <row r="27" spans="1:4">
+      <c r="A27" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
-      <c r="A26" s="2" t="s">
+    <row r="28" spans="1:4">
+      <c r="A28" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:1">
-      <c r="A27" s="2" t="s">
+    <row r="29" spans="1:4">
+      <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:1">
-      <c r="A28" s="2" t="s">
+    <row r="30" spans="1:4">
+      <c r="A30" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:1">
-      <c r="A29" s="2" t="s">
+    <row r="31" spans="1:4">
+      <c r="A31" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:1">
-      <c r="A30" s="2" t="s">
+    <row r="32" spans="1:4">
+      <c r="A32" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:1">
-      <c r="A31" s="2" t="s">
+    <row r="34" spans="1:1" ht="18">
+      <c r="A34" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="18">
-      <c r="A33" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1">
-      <c r="A34" s="2"/>
-    </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A35" s="2"/>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="18">
+      <c r="A41" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="18">
-      <c r="A40" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1">
-      <c r="A41" s="2"/>
-    </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="2" t="s">
-        <v>31</v>
-      </c>
+      <c r="A42" s="2"/>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="18">
+      <c r="A47" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:1" ht="18">
-      <c r="A46" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1">
-      <c r="A47" s="2"/>
-    </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="A48" s="2"/>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="18">
+      <c r="A53" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" spans="1:1" ht="18">
-      <c r="A52" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1">
-      <c r="A53" s="2"/>
-    </row>
     <row r="54" spans="1:1">
-      <c r="A54" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="A54" s="2"/>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="18">
+      <c r="A58" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="1:1" ht="18">
-      <c r="A57" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1">
-      <c r="A58" s="2"/>
-    </row>
     <row r="59" spans="1:1">
-      <c r="A59" s="2" t="s">
-        <v>42</v>
-      </c>
+      <c r="A59" s="2"/>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" ht="18">
+      <c r="A63" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="62" spans="1:1" ht="18">
-      <c r="A62" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1">
-      <c r="A63" s="2"/>
-    </row>
     <row r="64" spans="1:1">
-      <c r="A64" s="2" t="s">
-        <v>45</v>
-      </c>
+      <c r="A64" s="2"/>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="67" spans="1:1">
       <c r="A67" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="18">
+      <c r="A73" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="72" spans="1:1" ht="18">
-      <c r="A72" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1">
-      <c r="A73" s="2"/>
-    </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="A74" s="2"/>
     </row>
     <row r="75" spans="1:1">
       <c r="A75" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="76" spans="1:1">
       <c r="A76" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="77" spans="1:1">
       <c r="A77" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" ht="18">
+      <c r="A80" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="79" spans="1:1" ht="18">
-      <c r="A79" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1">
-      <c r="A80" s="2"/>
-    </row>
     <row r="81" spans="1:1">
-      <c r="A81" s="2" t="s">
-        <v>58</v>
-      </c>
+      <c r="A81" s="2"/>
     </row>
     <row r="82" spans="1:1">
       <c r="A82" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="83" spans="1:1">
       <c r="A83" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" ht="18">
+      <c r="A86" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="85" spans="1:1" ht="18">
-      <c r="A85" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1">
-      <c r="A86" s="2"/>
-    </row>
     <row r="87" spans="1:1">
-      <c r="A87" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="A87" s="2"/>
     </row>
     <row r="88" spans="1:1">
       <c r="A88" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="89" spans="1:1">
       <c r="A89" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>